<commit_message>
Update excel to design db
</commit_message>
<xml_diff>
--- a/Database/Quick-Design-Database.xlsx
+++ b/Database/Quick-Design-Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\Personal-Portfolio-Tracker-Website-V2\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCADDC9C-9FF3-4F61-9FDB-06315E13CE80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64C37A0C-54E9-4C7C-88C6-28E2239C9B06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{4E702879-61F5-4548-BD30-BE2863FD3951}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{4E702879-61F5-4548-BD30-BE2863FD3951}"/>
   </bookViews>
   <sheets>
     <sheet name="AuditLogs" sheetId="3" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="151">
   <si>
     <t>ID</t>
   </si>
@@ -130,9 +130,6 @@
     <t>Thời gian cập nhật tài khoản</t>
   </si>
   <si>
-    <t>Thời gian đăng nhập lần cuối</t>
-  </si>
-  <si>
     <t>Đã được kích hoạt hay chưa?</t>
   </si>
   <si>
@@ -154,9 +151,6 @@
     <t>Currency</t>
   </si>
   <si>
-    <t>char(3)</t>
-  </si>
-  <si>
     <t>varchar(10)</t>
   </si>
   <si>
@@ -166,9 +160,6 @@
     <t>INVEST, CASH, BANK, SAVINGS</t>
   </si>
   <si>
-    <t>VND, UST</t>
-  </si>
-  <si>
     <t>Not null, Default = (sysdatetime())</t>
   </si>
   <si>
@@ -181,9 +172,6 @@
     <t>Tiền trong account đầu tư (tiền gốc đã đầu tư)</t>
   </si>
   <si>
-    <t>Text</t>
-  </si>
-  <si>
     <t>Ghi chú</t>
   </si>
   <si>
@@ -229,9 +217,6 @@
     <t>Description</t>
   </si>
   <si>
-    <t>text</t>
-  </si>
-  <si>
     <t>AuditLogs</t>
   </si>
   <si>
@@ -491,6 +476,24 @@
   </si>
   <si>
     <t>decimal(18, 10)</t>
+  </si>
+  <si>
+    <t>nvarchar(MAX)</t>
+  </si>
+  <si>
+    <t>nvarchar(1000)</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Ngày tạo (luôn là server time tránh tình trạng các user ở khac timezone -&gt; lệch sort)</t>
+  </si>
+  <si>
+    <t>Thời gian đăng nhập lần cuối (chỉ lưu khi user thật sự login chứ không phải tạo mới).</t>
+  </si>
+  <si>
+    <t>VND, UST, USDT,… (để mở rộng sau này)</t>
   </si>
 </sst>
 </file>
@@ -551,7 +554,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -569,32 +572,6 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -618,21 +595,21 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -960,13 +937,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
+      <c r="A1" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -999,7 +976,7 @@
         <v>23</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1007,16 +984,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>33</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -1024,16 +1001,16 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>24</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -1041,7 +1018,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>5</v>
@@ -1050,7 +1027,7 @@
         <v>24</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -1058,16 +1035,16 @@
         <v>5</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>24</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -1075,16 +1052,16 @@
         <v>6</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>62</v>
+        <v>145</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>24</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -1092,16 +1069,16 @@
         <v>7</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>24</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -1109,7 +1086,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>15</v>
@@ -1118,7 +1095,7 @@
         <v>24</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -1126,16 +1103,16 @@
         <v>9</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>46</v>
+        <v>146</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>24</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -1152,7 +1129,7 @@
         <v>26</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -1172,18 +1149,18 @@
     <col min="2" max="2" width="15.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="48.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="84.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -1216,7 +1193,7 @@
         <v>23</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1279,7 +1256,7 @@
         <v>17</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>27</v>
@@ -1296,7 +1273,7 @@
         <v>17</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>28</v>
@@ -1312,11 +1289,9 @@
       <c r="C9" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="5" t="s">
-        <v>42</v>
-      </c>
+      <c r="D9" s="5"/>
       <c r="E9" s="5" t="s">
-        <v>29</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -1333,7 +1308,7 @@
         <v>26</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -1344,11 +1319,11 @@
         <v>4</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>46</v>
+        <v>146</v>
       </c>
       <c r="D11" s="5"/>
       <c r="E11" s="5" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -1365,7 +1340,7 @@
         <v>26</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -1381,22 +1356,22 @@
   <dimension ref="A1:F15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.85546875" style="8" customWidth="1"/>
-    <col min="2" max="2" width="19.5703125" style="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="69" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="8"/>
+    <col min="1" max="1" width="3.85546875" style="7" customWidth="1"/>
+    <col min="2" max="2" width="19.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="69" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
+      <c r="A1" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
     </row>
     <row r="2" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -1429,7 +1404,7 @@
         <v>23</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
@@ -1437,19 +1412,19 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="3" t="s">
-        <v>34</v>
-      </c>
       <c r="F4" s="9" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
@@ -1457,7 +1432,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>15</v>
@@ -1466,7 +1441,7 @@
         <v>24</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F5" s="9"/>
     </row>
@@ -1478,13 +1453,13 @@
         <v>2</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>24</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
@@ -1492,14 +1467,14 @@
         <v>5</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="D7" s="5"/>
       <c r="E7" s="5" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
@@ -1507,16 +1482,16 @@
         <v>6</v>
       </c>
       <c r="B8" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>36</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>37</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>24</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>41</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
@@ -1524,14 +1499,14 @@
         <v>7</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="5" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
@@ -1539,14 +1514,14 @@
         <v>8</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="5" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
@@ -1554,16 +1529,16 @@
         <v>9</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>24</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
@@ -1577,10 +1552,10 @@
         <v>17</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
@@ -1594,10 +1569,10 @@
         <v>17</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
@@ -1608,11 +1583,11 @@
         <v>4</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>46</v>
+        <v>146</v>
       </c>
       <c r="D14" s="5"/>
       <c r="E14" s="5" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
@@ -1629,7 +1604,7 @@
         <v>26</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -1655,13 +1630,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
+      <c r="A1" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -1694,7 +1669,7 @@
         <v>23</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1702,16 +1677,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -1719,16 +1694,16 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>24</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -1736,16 +1711,16 @@
         <v>4</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>24</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -1759,10 +1734,10 @@
         <v>17</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -1779,12 +1754,12 @@
         <v>26</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
     <row r="17" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E17" s="6" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1809,13 +1784,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
+      <c r="A1" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -1848,7 +1823,7 @@
         <v>23</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1856,16 +1831,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D4" s="11" t="s">
         <v>25</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -1873,14 +1848,16 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="D5" s="12"/>
+        <v>69</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>24</v>
+      </c>
       <c r="E5" s="5" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -1891,13 +1868,13 @@
         <v>16</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -1908,13 +1885,13 @@
         <v>18</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -1928,16 +1905,15 @@
         <v>7</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="D4:D5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1945,25 +1921,25 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71E1E830-2449-4402-A0A1-B6CC77BF2E77}">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="38.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="44" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
+      <c r="A1" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -1996,7 +1972,7 @@
         <v>23</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -2004,16 +1980,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="D4" s="10" t="s">
         <v>25</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -2021,14 +1997,14 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="D5" s="10"/>
       <c r="E5" s="5" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -2036,16 +2012,16 @@
         <v>4</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -2053,16 +2029,16 @@
         <v>5</v>
       </c>
       <c r="B7" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="E7" s="5" t="s">
         <v>89</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -2070,16 +2046,16 @@
         <v>6</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>70</v>
+        <v>36</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>71</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -2087,16 +2063,16 @@
         <v>7</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>95</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -2104,16 +2080,33 @@
         <v>8</v>
       </c>
       <c r="B10" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="3">
+        <v>9</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C11" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>68</v>
+      <c r="D11" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -2139,13 +2132,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
+      <c r="A1" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -2178,7 +2171,7 @@
         <v>23</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -2186,16 +2179,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -2203,14 +2196,14 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D5" s="10"/>
       <c r="E5" s="5" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -2218,16 +2211,16 @@
         <v>4</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -2235,16 +2228,16 @@
         <v>5</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -2252,16 +2245,16 @@
         <v>6</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -2269,14 +2262,14 @@
         <v>7</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="5" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -2284,14 +2277,14 @@
         <v>8</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="5" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -2305,10 +2298,10 @@
         <v>17</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -2322,10 +2315,10 @@
         <v>17</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -2336,11 +2329,11 @@
         <v>4</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>46</v>
+        <v>145</v>
       </c>
       <c r="D13" s="5"/>
       <c r="E13" s="5" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -2354,10 +2347,10 @@
         <v>7</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -2371,7 +2364,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56BD71B3-84EC-4007-9128-7454E75BD5E5}">
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -2383,13 +2376,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
+      <c r="A1" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -2422,313 +2415,332 @@
         <v>23</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>77</v>
+      <c r="B4" s="11" t="s">
+        <v>72</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>83</v>
+      <c r="D4" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>3</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>79</v>
+      <c r="B5" s="11" t="s">
+        <v>74</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>92</v>
+      <c r="D5" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>4</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="D6" s="5" t="s">
+      <c r="B6" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="D6" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="5" t="s">
-        <v>110</v>
+      <c r="E6" s="11" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>5</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5" t="s">
-        <v>115</v>
+      <c r="B7" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>6</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5" t="s">
-        <v>116</v>
+      <c r="B8" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>7</v>
       </c>
-      <c r="B9" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5" t="s">
-        <v>147</v>
+      <c r="B9" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>8</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5" t="s">
-        <v>122</v>
+      <c r="B10" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>9</v>
       </c>
-      <c r="B11" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5" t="s">
-        <v>142</v>
+      <c r="B11" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>10</v>
       </c>
-      <c r="B12" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5" t="s">
-        <v>117</v>
+      <c r="B12" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>11</v>
       </c>
-      <c r="B13" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5" t="s">
-        <v>143</v>
+      <c r="B13" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>12</v>
       </c>
-      <c r="B14" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5" t="s">
-        <v>148</v>
+      <c r="B14" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>13</v>
       </c>
-      <c r="B15" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>118</v>
+      <c r="B15" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>14</v>
       </c>
-      <c r="B16" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5" t="s">
-        <v>139</v>
+      <c r="B16" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>15</v>
       </c>
-      <c r="B17" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5" t="s">
-        <v>138</v>
+      <c r="B17" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>16</v>
       </c>
-      <c r="B18" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="D18" s="5" t="s">
+      <c r="B18" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="D18" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="E18" s="5" t="s">
-        <v>119</v>
+      <c r="E18" s="11" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>17</v>
       </c>
-      <c r="B19" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="D19" s="5" t="s">
+      <c r="B19" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="D19" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="E19" s="5" t="s">
-        <v>120</v>
+      <c r="E19" s="11" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>18</v>
       </c>
-      <c r="B20" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="D20" s="5" t="s">
+      <c r="B20" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="D20" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="E20" s="5" t="s">
-        <v>121</v>
+      <c r="E20" s="11" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>19</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C21" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C21" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="33" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>20</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="D22" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="3">
         <v>21</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="B23" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C23" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="D23" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="E22" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E31" s="6" t="s">
-        <v>78</v>
+      <c r="E23" s="11" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E32" s="6" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Generate script using SQL Server
</commit_message>
<xml_diff>
--- a/Database/Quick-Design-Database.xlsx
+++ b/Database/Quick-Design-Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\Personal-Portfolio-Tracker-Website-V2\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64C37A0C-54E9-4C7C-88C6-28E2239C9B06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7873676-78CF-42DD-A5E7-F60DD15FF750}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{4E702879-61F5-4548-BD30-BE2863FD3951}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{4E702879-61F5-4548-BD30-BE2863FD3951}"/>
   </bookViews>
   <sheets>
     <sheet name="AuditLogs" sheetId="3" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="153">
   <si>
     <t>ID</t>
   </si>
@@ -301,9 +301,6 @@
     <t>varchar(100)</t>
   </si>
   <si>
-    <t>Not null, Default  0</t>
-  </si>
-  <si>
     <t>Mã ticker</t>
   </si>
   <si>
@@ -494,6 +491,15 @@
   </si>
   <si>
     <t>VND, UST, USDT,… (để mở rộng sau này)</t>
+  </si>
+  <si>
+    <t>Not null, Default = 0, &gt;0</t>
+  </si>
+  <si>
+    <t>varchar(200)</t>
+  </si>
+  <si>
+    <t>Not null, (CONVERT(date, sysdatetime()))</t>
   </si>
 </sst>
 </file>
@@ -596,6 +602,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -604,12 +616,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -937,13 +943,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -976,7 +982,7 @@
         <v>23</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1055,7 +1061,7 @@
         <v>57</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>24</v>
@@ -1069,7 +1075,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>65</v>
@@ -1078,7 +1084,7 @@
         <v>24</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -1086,7 +1092,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>15</v>
@@ -1095,7 +1101,7 @@
         <v>24</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -1103,16 +1109,16 @@
         <v>9</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>24</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -1154,13 +1160,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -1193,7 +1199,7 @@
         <v>23</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1291,7 +1297,7 @@
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -1319,7 +1325,7 @@
         <v>4</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D11" s="5"/>
       <c r="E11" s="5" t="s">
@@ -1365,13 +1371,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
     </row>
     <row r="2" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -1404,7 +1410,7 @@
         <v>23</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
@@ -1423,7 +1429,7 @@
       <c r="E4" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="11" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1443,7 +1449,7 @@
       <c r="E5" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="F5" s="9"/>
+      <c r="F5" s="11"/>
     </row>
     <row r="6" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
@@ -1491,7 +1497,7 @@
         <v>24</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
@@ -1502,9 +1508,11 @@
         <v>49</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="D9" s="5"/>
+        <v>126</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>150</v>
+      </c>
       <c r="E9" s="5" t="s">
         <v>42</v>
       </c>
@@ -1517,9 +1525,11 @@
         <v>45</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="D10" s="5"/>
+        <v>126</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>150</v>
+      </c>
       <c r="E10" s="5" t="s">
         <v>51</v>
       </c>
@@ -1532,10 +1542,10 @@
         <v>50</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>24</v>
+        <v>150</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>52</v>
@@ -1583,7 +1593,7 @@
         <v>4</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D14" s="5"/>
       <c r="E14" s="5" t="s">
@@ -1630,13 +1640,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -1669,7 +1679,7 @@
         <v>23</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1714,10 +1724,10 @@
         <v>50</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>24</v>
+        <v>150</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>52</v>
@@ -1784,13 +1794,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -1823,7 +1833,7 @@
         <v>23</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1836,7 +1846,7 @@
       <c r="C4" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E4" s="5" t="s">
@@ -1853,7 +1863,7 @@
       <c r="C5" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="8" t="s">
         <v>24</v>
       </c>
       <c r="E5" s="5" t="s">
@@ -1891,7 +1901,7 @@
         <v>39</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -1933,13 +1943,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -1972,7 +1982,7 @@
         <v>23</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1980,16 +1990,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>25</v>
+        <v>124</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>32</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>99</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -1997,14 +2007,16 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>34</v>
+        <v>77</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="D5" s="10"/>
+        <v>55</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>25</v>
+      </c>
       <c r="E5" s="5" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -2012,16 +2024,16 @@
         <v>4</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>24</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>126</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -2032,13 +2044,13 @@
         <v>84</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -2055,7 +2067,7 @@
         <v>24</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -2089,7 +2101,7 @@
         <v>39</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -2103,16 +2115,15 @@
         <v>7</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>86</v>
+        <v>26</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>63</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="D4:D5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2132,13 +2143,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -2171,7 +2182,7 @@
         <v>23</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -2184,8 +2195,8 @@
       <c r="C4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="10" t="s">
-        <v>104</v>
+      <c r="D4" s="12" t="s">
+        <v>103</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>78</v>
@@ -2201,9 +2212,9 @@
       <c r="C5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="10"/>
+      <c r="D5" s="12"/>
       <c r="E5" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -2211,16 +2222,16 @@
         <v>4</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D6" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>92</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -2228,16 +2239,16 @@
         <v>5</v>
       </c>
       <c r="B7" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="E7" s="5" t="s">
         <v>95</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -2245,16 +2256,16 @@
         <v>6</v>
       </c>
       <c r="B8" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>97</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -2262,14 +2273,14 @@
         <v>7</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -2277,14 +2288,14 @@
         <v>8</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -2318,7 +2329,7 @@
         <v>39</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -2329,7 +2340,7 @@
         <v>4</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D13" s="5"/>
       <c r="E13" s="5" t="s">
@@ -2347,7 +2358,7 @@
         <v>7</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>86</v>
+        <v>26</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>63</v>
@@ -2370,19 +2381,19 @@
     <col min="1" max="1" width="3.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="44.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="69.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -2415,23 +2426,23 @@
         <v>23</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>2</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="8" t="s">
         <v>72</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="8" t="s">
         <v>78</v>
       </c>
     </row>
@@ -2439,268 +2450,268 @@
       <c r="A5" s="3">
         <v>3</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="8" t="s">
         <v>74</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="11" t="s">
-        <v>87</v>
+      <c r="E5" s="8" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>4</v>
       </c>
-      <c r="B6" s="11" t="s">
-        <v>139</v>
-      </c>
-      <c r="C6" s="11" t="s">
+      <c r="B6" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="11" t="s">
-        <v>105</v>
+      <c r="E6" s="8" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>5</v>
       </c>
-      <c r="B7" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>127</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>110</v>
+      <c r="B7" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>6</v>
       </c>
-      <c r="B8" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>127</v>
-      </c>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11" t="s">
-        <v>111</v>
+      <c r="B8" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>7</v>
       </c>
-      <c r="B9" s="11" t="s">
-        <v>140</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>127</v>
-      </c>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11" t="s">
-        <v>142</v>
+      <c r="B9" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>8</v>
       </c>
-      <c r="B10" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>127</v>
-      </c>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11" t="s">
-        <v>117</v>
+      <c r="B10" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>9</v>
       </c>
-      <c r="B11" s="11" t="s">
-        <v>135</v>
-      </c>
-      <c r="C11" s="11" t="s">
-        <v>144</v>
-      </c>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11" t="s">
-        <v>137</v>
+      <c r="B11" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>10</v>
       </c>
-      <c r="B12" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>127</v>
-      </c>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11" t="s">
-        <v>112</v>
+      <c r="B12" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>11</v>
       </c>
-      <c r="B13" s="11" t="s">
-        <v>136</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>144</v>
-      </c>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11" t="s">
-        <v>138</v>
+      <c r="B13" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>12</v>
       </c>
-      <c r="B14" s="11" t="s">
-        <v>141</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>127</v>
-      </c>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B14" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>13</v>
       </c>
-      <c r="B15" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="C15" s="11" t="s">
-        <v>147</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>113</v>
+      <c r="B15" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>14</v>
       </c>
-      <c r="B16" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="C16" s="11" t="s">
-        <v>127</v>
-      </c>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11" t="s">
-        <v>134</v>
+      <c r="B16" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>15</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8" t="s">
         <v>132</v>
-      </c>
-      <c r="C17" s="11" t="s">
-        <v>144</v>
-      </c>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>16</v>
       </c>
-      <c r="B18" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="C18" s="11" t="s">
+      <c r="B18" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="D18" s="11" t="s">
+      <c r="C18" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="D18" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="E18" s="11" t="s">
-        <v>114</v>
+      <c r="E18" s="8" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>17</v>
       </c>
-      <c r="B19" s="11" t="s">
-        <v>129</v>
-      </c>
-      <c r="C19" s="11" t="s">
-        <v>127</v>
-      </c>
-      <c r="D19" s="11" t="s">
+      <c r="B19" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="D19" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="E19" s="11" t="s">
-        <v>115</v>
+      <c r="E19" s="8" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>18</v>
       </c>
-      <c r="B20" s="11" t="s">
-        <v>130</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>127</v>
-      </c>
-      <c r="D20" s="11" t="s">
+      <c r="B20" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="D20" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="E20" s="11" t="s">
-        <v>116</v>
+      <c r="E20" s="8" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>19</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="C21" s="11" t="s">
-        <v>146</v>
-      </c>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11" t="s">
+      <c r="C21" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8" t="s">
         <v>43</v>
       </c>
     </row>
@@ -2708,33 +2719,33 @@
       <c r="A22" s="3">
         <v>20</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="D22" s="11" t="s">
+      <c r="D22" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="E22" s="12" t="s">
-        <v>148</v>
+      <c r="E22" s="9" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>21</v>
       </c>
-      <c r="B23" s="11" t="s">
+      <c r="B23" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C23" s="11" t="s">
+      <c r="C23" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D23" s="11" t="s">
+      <c r="D23" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="E23" s="11" t="s">
+      <c r="E23" s="8" t="s">
         <v>63</v>
       </c>
     </row>

</xml_diff>